<commit_message>
Fix question context in Reading2.xlsx: bound windows to prev/next question markers
Agent-Logs-Url: https://github.com/academiaohara/cambridge-exams/sessions/d0bba03e-657f-484e-8fe3-fcd101822625

Co-authored-by: academiaohara <253255719+academiaohara@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/social media/B2/Reading2.xlsx
+++ b/social media/B2/Reading2.xlsx
@@ -28,10 +28,9 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="10"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -41,13 +40,16 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="004472C4"/>
-        <bgColor rgb="004472C4"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00EBF0FB"/>
-        <bgColor rgb="00EBF0FB"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
   </fills>
@@ -71,7 +73,7 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -469,7 +471,7 @@
     <col width="45" customWidth="1" min="25" max="25"/>
   </cols>
   <sheetData>
-    <row r="1" ht="25" customHeight="1">
+    <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>ID</t>
@@ -596,48 +598,48 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="60" customHeight="1">
+    <row r="2">
       <c r="A2" s="2" t="n">
         <v>1</v>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>...Snowy mountain peaks serve as a backdrop to crystal-clear lakes surrounded by green forests. Once a major trade route (9) between India and Tibet, Pokhara is Nepal’s second largest city. There are three main lakes in the area, (10) the most...</t>
+          <t>...Snowy mountain peaks serve as a backdrop to crystal-clear lakes surrounded by green forests. Once a major trade route (9) between India and Tibet, Pokhara is Nepal’s second largest city. There are three main lakes in the area,...</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>...route (9) between India and Tibet, Pokhara is Nepal’s second largest city. There are three main lakes in the area, (10) the most popular of (11) which is Phewa Lake. Tourists come here (12) in their thousands to admire the mirror-like...</t>
+          <t>...between India and Tibet, Pokhara is Nepal’s second largest city. There are three main lakes in the area, (10) the most popular of...</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>...and Tibet, Pokhara is Nepal’s second largest city. There are three main lakes in the area, (10) the most popular of (11) which is Phewa Lake. Tourists come here (12) in their thousands to admire the mirror-like waters and relax amongst...</t>
+          <t>...the most popular of (11) which is Phewa Lake. Tourists come here...</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>...city. There are three main lakes in the area, (10) the most popular of (11) which is Phewa Lake. Tourists come here (12) in their thousands to admire the mirror-like waters and relax amongst some truly spectacular scenery. Lakeside, a...</t>
+          <t>...which is Phewa Lake. Tourists come here (12) in their thousands to admire the mirror-like waters and relax amongst some truly spectacular scenery. Lakeside, a...</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>...to admire the mirror-like waters and relax amongst some truly spectacular scenery. Lakeside, a thriving resort town, (13) has emerged along the eastern shore of the lake and offers visitors (14) a wealth of hotels, restaurants and souvenir...</t>
+          <t>...to admire the mirror-like waters and relax amongst some truly spectacular scenery. Lakeside, a thriving resort town, (13) has emerged along the eastern shore of the lake and offers visitors...</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>...scenery. Lakeside, a thriving resort town, (13) has emerged along the eastern shore of the lake and offers visitors (14) a wealth of hotels, restaurants and souvenir shops. For those (15) who want to get out and explore the countryside,...</t>
+          <t>...has emerged along the eastern shore of the lake and offers visitors (14) a wealth of hotels, restaurants and souvenir shops. For those...</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>...the eastern shore of the lake and offers visitors (14) a wealth of hotels, restaurants and souvenir shops. For those (15) who want to get out and explore the countryside, bikes can (16) be hired to explore the lush green fields and the...</t>
+          <t>...a wealth of hotels, restaurants and souvenir shops. For those (15) who want to get out and explore the countryside, bikes can...</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>...of hotels, restaurants and souvenir shops. For those (15) who want to get out and explore the countryside, bikes can (16) be hired to explore the lush green fields and the gorgeous little villages or to cycle along river banks. Visitors can...</t>
+          <t>...who want to get out and explore the countryside, bikes can (16) be hired to explore the lush green fields and the gorgeous little villages or to cycle along river banks. Visitors can...</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
@@ -721,48 +723,48 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="60" customHeight="1">
+    <row r="3">
       <c r="A3" s="3" t="n">
         <v>2</v>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>...an area of over 5.5 million square kilometres and spans across nine countries in South America. The rainforest is home (9) to an incredible diversity of wildlife, with scientists estimating that millions of species (10) of insects, plants...</t>
+          <t>...an area of over 5.5 million square kilometres and spans across nine countries in South America. The rainforest is home (9) to an incredible diversity of wildlife, with scientists estimating that millions of species...</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>...The rainforest is home (9) to an incredible diversity of wildlife, with scientists estimating that millions of species (10) of insects, plants and animals live within its boundaries. Many of these species have (11) not yet been discovered or...</t>
+          <t>...to an incredible diversity of wildlife, with scientists estimating that millions of species (10) of insects, plants and animals live within its boundaries. Many of these species have...</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>...that millions of species (10) of insects, plants and animals live within its boundaries. Many of these species have (11) not yet been discovered or documented by researchers. The Amazon River, (12) which flows through the heart of the...</t>
+          <t>...of insects, plants and animals live within its boundaries. Many of these species have (11) not yet been discovered or documented by researchers. The Amazon River,...</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>...boundaries. Many of these species have (11) not yet been discovered or documented by researchers. The Amazon River, (12) which flows through the heart of the rainforest, is the second longest river in the world. Unfortunately,...</t>
+          <t>...not yet been discovered or documented by researchers. The Amazon River, (12) which flows through the heart of the rainforest, is the second longest river in the world. Unfortunately,...</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>...flows through the heart of the rainforest, is the second longest river in the world. Unfortunately, deforestation (13) has become a serious threat to this precious ecosystem. Every year, thousands of square kilometres (14) are cleared...</t>
+          <t>...flows through the heart of the rainforest, is the second longest river in the world. Unfortunately, deforestation (13) has become a serious threat to this precious ecosystem. Every year, thousands of square kilometres...</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>...deforestation (13) has become a serious threat to this precious ecosystem. Every year, thousands of square kilometres (14) are cleared for agriculture and logging. Conservation groups are working hard to protect (15) the rainforest, but they...</t>
+          <t>...has become a serious threat to this precious ecosystem. Every year, thousands of square kilometres (14) are cleared for agriculture and logging. Conservation groups are working hard to protect...</t>
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>...of square kilometres (14) are cleared for agriculture and logging. Conservation groups are working hard to protect (15) the rainforest, but they face many challenges. (16) If we don't take action soon, future generations may never...</t>
+          <t>...are cleared for agriculture and logging. Conservation groups are working hard to protect (15) the rainforest, but they face many challenges....</t>
         </is>
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>...and logging. Conservation groups are working hard to protect (15) the rainforest, but they face many challenges. (16) If we don't take action soon, future generations may never experience the wonder of this natural treasure.</t>
+          <t>...the rainforest, but they face many challenges. (16) If we don't take action soon, future generations may never experience the wonder of this natural treasure.</t>
         </is>
       </c>
       <c r="J3" s="3" t="inlineStr">
@@ -846,7 +848,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="60" customHeight="1">
+    <row r="4">
       <c r="A4" s="2" t="n">
         <v>3</v>
       </c>
@@ -857,37 +859,37 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>...his goats became energetic after eating berries from a certain tree. He tried the berries himself and experienced (10) the same effect. The knowledge of coffee soon spread to the Arabian Peninsula, (11) where it was cultivated and...</t>
+          <t>...his goats became energetic after eating berries from a certain tree. He tried the berries himself and experienced (10) the same effect. The knowledge of coffee soon spread to the Arabian Peninsula,...</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>...berries himself and experienced (10) the same effect. The knowledge of coffee soon spread to the Arabian Peninsula, (11) where it was cultivated and traded. By the 15th century, coffee (12) was being grown in Yemen, and coffee houses began...</t>
+          <t>...the same effect. The knowledge of coffee soon spread to the Arabian Peninsula, (11) where it was cultivated and traded. By the 15th century, coffee...</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>...of coffee soon spread to the Arabian Peninsula, (11) where it was cultivated and traded. By the 15th century, coffee (12) was being grown in Yemen, and coffee houses began to appear throughout the Middle East. Coffee arrived in Europe...</t>
+          <t>...where it was cultivated and traded. By the 15th century, coffee (12) was being grown in Yemen, and coffee houses began to appear throughout the Middle East. Coffee arrived in Europe...</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>...to appear throughout the Middle East. Coffee arrived in Europe during the 17th century and quickly gained popularity, (13) despite some initial resistance from religious authorities. Today, coffee is grown in over 70 countries, (14) with...</t>
+          <t>...to appear throughout the Middle East. Coffee arrived in Europe during the 17th century and quickly gained popularity, (13) despite some initial resistance from religious authorities. Today, coffee is grown in over 70 countries,...</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>...(13) despite some initial resistance from religious authorities. Today, coffee is grown in over 70 countries, (14) with Brazil being the largest producer. Whether you prefer it black (15) or with milk, there's no denying that coffee...</t>
+          <t>...despite some initial resistance from religious authorities. Today, coffee is grown in over 70 countries, (14) with Brazil being the largest producer. Whether you prefer it black...</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>...Today, coffee is grown in over 70 countries, (14) with Brazil being the largest producer. Whether you prefer it black (15) or with milk, there's no denying that coffee (16) has become an essential part of modern life for many people around...</t>
+          <t>...with Brazil being the largest producer. Whether you prefer it black (15) or with milk, there's no denying that coffee...</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>...with Brazil being the largest producer. Whether you prefer it black (15) or with milk, there's no denying that coffee (16) has become an essential part of modern life for many people around the globe.</t>
+          <t>...or with milk, there's no denying that coffee (16) has become an essential part of modern life for many people around the globe.</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
@@ -971,23 +973,23 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="60" customHeight="1">
+    <row r="5">
       <c r="A5" s="3" t="n">
         <v>4</v>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>...cultivating food in urban environments, such as on rooftops, in community gardens, or even inside buildings. One (9) of the main benefits of urban farming is that it reduces the distance food travels from farm to plate, (10) which...</t>
+          <t>...cultivating food in urban environments, such as on rooftops, in community gardens, or even inside buildings. One (9) of the main benefits of urban farming is that it reduces the distance food travels from farm to plate,...</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>...One (9) of the main benefits of urban farming is that it reduces the distance food travels from farm to plate, (10) which means produce is fresher and has a smaller carbon footprint. Urban farms can (11) also provide green spaces in...</t>
+          <t>...of the main benefits of urban farming is that it reduces the distance food travels from farm to plate, (10) which means produce is fresher and has a smaller carbon footprint. Urban farms can...</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>...travels from farm to plate, (10) which means produce is fresher and has a smaller carbon footprint. Urban farms can (11) also provide green spaces in concrete jungles, improving air quality and creating habitats for wildlife. Many cities...</t>
+          <t>...which means produce is fresher and has a smaller carbon footprint. Urban farms can (11) also provide green spaces in concrete jungles, improving air quality and creating habitats for wildlife. Many cities...</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
@@ -997,22 +999,22 @@
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>...to community groups. However, urban farming does face challenges. Space is limited in cities, and the cost of land can (13) be very high. Despite these difficulties, creative solutions (14) are being developed, such as vertical farming and...</t>
+          <t>...to community groups. However, urban farming does face challenges. Space is limited in cities, and the cost of land can (13) be very high. Despite these difficulties, creative solutions...</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>...Space is limited in cities, and the cost of land can (13) be very high. Despite these difficulties, creative solutions (14) are being developed, such as vertical farming and hydroponic systems. These innovations allow food to be grown (15) in...</t>
+          <t>...be very high. Despite these difficulties, creative solutions (14) are being developed, such as vertical farming and hydroponic systems. These innovations allow food to be grown...</t>
         </is>
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>...(14) are being developed, such as vertical farming and hydroponic systems. These innovations allow food to be grown (15) in smaller spaces using less water. (16) As cities continue to expand, urban farming may become an essential part of...</t>
+          <t>...are being developed, such as vertical farming and hydroponic systems. These innovations allow food to be grown (15) in smaller spaces using less water....</t>
         </is>
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>...farming and hydroponic systems. These innovations allow food to be grown (15) in smaller spaces using less water. (16) As cities continue to expand, urban farming may become an essential part of feeding growing populations.</t>
+          <t>...in smaller spaces using less water. (16) As cities continue to expand, urban farming may become an essential part of feeding growing populations.</t>
         </is>
       </c>
       <c r="J5" s="3" t="inlineStr">
@@ -1096,33 +1098,33 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="60" customHeight="1">
+    <row r="6">
       <c r="A6" s="2" t="n">
         <v>5</v>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>...light appear in the night sky near the Arctic Circle and have fascinated people for centuries. The phenomenon occurs (9) when charged particles from the sun collide with gases in Earth's atmosphere. The colours you see depend (10) on which...</t>
+          <t>...light appear in the night sky near the Arctic Circle and have fascinated people for centuries. The phenomenon occurs (9) when charged particles from the sun collide with gases in Earth's atmosphere. The colours you see depend...</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>...occurs (9) when charged particles from the sun collide with gases in Earth's atmosphere. The colours you see depend (10) on which gas is involved: oxygen produces green and red lights, (11) while nitrogen creates blue and purple hues. The...</t>
+          <t>...when charged particles from the sun collide with gases in Earth's atmosphere. The colours you see depend (10) on which gas is involved: oxygen produces green and red lights,...</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>...in Earth's atmosphere. The colours you see depend (10) on which gas is involved: oxygen produces green and red lights, (11) while nitrogen creates blue and purple hues. The best time to witness this natural wonder is (12) during the winter...</t>
+          <t>...on which gas is involved: oxygen produces green and red lights, (11) while nitrogen creates blue and purple hues. The best time to witness this natural wonder is...</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>...and red lights, (11) while nitrogen creates blue and purple hues. The best time to witness this natural wonder is (12) during the winter months, when nights are long and dark. Countries such (13) as Norway, Iceland, and Canada offer some...</t>
+          <t>...while nitrogen creates blue and purple hues. The best time to witness this natural wonder is (12) during the winter months, when nights are long and dark. Countries such...</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>...time to witness this natural wonder is (12) during the winter months, when nights are long and dark. Countries such (13) as Norway, Iceland, and Canada offer some of the best viewing opportunities. However, seeing the Northern Lights is...</t>
+          <t>...during the winter months, when nights are long and dark. Countries such (13) as Norway, Iceland, and Canada offer some of the best viewing opportunities. However, seeing the Northern Lights is...</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -1132,12 +1134,12 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>...since solar activity and weather conditions must both be favourable. Many tourists travel to the Arctic specifically (15) to experience this phenomenon. Those (16) who have witnessed it describe the experience as magical and unforgettable,...</t>
+          <t>...since solar activity and weather conditions must both be favourable. Many tourists travel to the Arctic specifically (15) to experience this phenomenon. Those...</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>...must both be favourable. Many tourists travel to the Arctic specifically (15) to experience this phenomenon. Those (16) who have witnessed it describe the experience as magical and unforgettable, with the lights appearing to dance across...</t>
+          <t>...to experience this phenomenon. Those (16) who have witnessed it describe the experience as magical and unforgettable, with the lights appearing to dance across...</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
@@ -1207,7 +1209,7 @@
       </c>
       <c r="W6" s="2" t="inlineStr">
         <is>
-          <t>Conjunction meaning 'because', used to introduce a reason. Both 'since' and 'as' can introduce a reason clause, making '...</t>
+          <t>Conjunction meaning 'because', used to introduce a reason. Both 'since' and 'as' can introduce a reason clause, making 'since' the expected answer here.</t>
         </is>
       </c>
       <c r="X6" s="2" t="inlineStr">
@@ -1221,7 +1223,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="60" customHeight="1">
+    <row r="7">
       <c r="A7" s="3" t="n">
         <v>6</v>
       </c>
@@ -1232,37 +1234,37 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>...a chemical called luciferin reacts with oxygen in the presence of an enzyme. Different species use bioluminescence (10) for different purposes: some use it to attract prey, (11) while others use it to communicate or find mates. In the...</t>
+          <t>...a chemical called luciferin reacts with oxygen in the presence of an enzyme. Different species use bioluminescence (10) for different purposes: some use it to attract prey,...</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>...presence of an enzyme. Different species use bioluminescence (10) for different purposes: some use it to attract prey, (11) while others use it to communicate or find mates. In the deep ocean, (12) where sunlight cannot reach, bioluminescence...</t>
+          <t>...for different purposes: some use it to attract prey, (11) while others use it to communicate or find mates. In the deep ocean,...</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>...purposes: some use it to attract prey, (11) while others use it to communicate or find mates. In the deep ocean, (12) where sunlight cannot reach, bioluminescence is particularly common, with up to 90% of deep-sea creatures possessing...</t>
+          <t>...while others use it to communicate or find mates. In the deep ocean, (12) where sunlight cannot reach, bioluminescence is particularly common, with up to 90% of deep-sea creatures possessing...</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>...up to 90% of deep-sea creatures possessing this ability. One of the most spectacular displays of bioluminescence can (13) be seen in certain coastal areas, where billions of tiny plankton light up the water at night. This creates (14) a...</t>
+          <t>...up to 90% of deep-sea creatures possessing this ability. One of the most spectacular displays of bioluminescence can (13) be seen in certain coastal areas, where billions of tiny plankton light up the water at night. This creates...</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>...can (13) be seen in certain coastal areas, where billions of tiny plankton light up the water at night. This creates (14) a magical blue glow that looks like something from a science fiction film. Scientists are now studying bioluminescence...</t>
+          <t>...be seen in certain coastal areas, where billions of tiny plankton light up the water at night. This creates (14) a magical blue glow that looks like something from a science fiction film. Scientists are now studying bioluminescence...</t>
         </is>
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
-          <t>...Scientists are now studying bioluminescence to develop new technologies, including more efficient lighting systems. (15) Although we have learned much about this phenomenon, there is still (16) much/a lot to discover about how and why...</t>
+          <t>...Scientists are now studying bioluminescence to develop new technologies, including more efficient lighting systems. (15) Although we have learned much about this phenomenon, there is still...</t>
         </is>
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>...including more efficient lighting systems. (15) Although we have learned much about this phenomenon, there is still (16) much/a lot to discover about how and why organisms produce light.</t>
+          <t>...Although we have learned much about this phenomenon, there is still (16) much/a lot to discover about how and why organisms produce light.</t>
         </is>
       </c>
       <c r="J7" s="3" t="inlineStr">
@@ -1346,7 +1348,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="60" customHeight="1">
+    <row r="8">
       <c r="A8" s="2" t="n">
         <v>7</v>
       </c>
@@ -1362,32 +1364,32 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>...reef, but rather a complex system made up of nearly 3,000 individual reefs and 900 islands. The Great Barrier Reef (11) has existed for millions of years, slowly built by tiny coral polyps over countless generations. Tourism plays (12) an...</t>
+          <t>...reef, but rather a complex system made up of nearly 3,000 individual reefs and 900 islands. The Great Barrier Reef (11) has existed for millions of years, slowly built by tiny coral polyps over countless generations. Tourism plays...</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>...(11) has existed for millions of years, slowly built by tiny coral polyps over countless generations. Tourism plays (12) an important role in the local economy, with millions of visitors coming each year to snorkel and dive. However, the...</t>
+          <t>...has existed for millions of years, slowly built by tiny coral polyps over countless generations. Tourism plays (12) an important role in the local economy, with millions of visitors coming each year to snorkel and dive. However, the...</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>...local economy, with millions of visitors coming each year to snorkel and dive. However, the reef faces serious threats (13) from climate change, pollution, and overfishing. Rising ocean temperatures (14) have caused widespread coral...</t>
+          <t>...local economy, with millions of visitors coming each year to snorkel and dive. However, the reef faces serious threats (13) from climate change, pollution, and overfishing. Rising ocean temperatures...</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>...the reef faces serious threats (13) from climate change, pollution, and overfishing. Rising ocean temperatures (14) have caused widespread coral bleaching, which occurs (15) when corals expel the algae living in their tissues....</t>
+          <t>...from climate change, pollution, and overfishing. Rising ocean temperatures (14) have caused widespread coral bleaching, which occurs...</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>...pollution, and overfishing. Rising ocean temperatures (14) have caused widespread coral bleaching, which occurs (15) when corals expel the algae living in their tissues. Scientists are working urgently to find solutions, (16) as the...</t>
+          <t>...have caused widespread coral bleaching, which occurs (15) when corals expel the algae living in their tissues. Scientists are working urgently to find solutions,...</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>...occurs (15) when corals expel the algae living in their tissues. Scientists are working urgently to find solutions, (16) as the loss of this ecosystem would be catastrophic for marine biodiversity.</t>
+          <t>...when corals expel the algae living in their tissues. Scientists are working urgently to find solutions, (16) as the loss of this ecosystem would be catastrophic for marine biodiversity.</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
@@ -1471,7 +1473,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="60" customHeight="1">
+    <row r="9">
       <c r="A9" s="3" t="n">
         <v>8</v>
       </c>
@@ -1492,12 +1494,12 @@
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>...Banksy, have achieved international fame despite remaining anonymous. Today, many cities actively encourage street art (12) by designating legal walls where artists can work freely. Today, street art has gained recognition and, (13) as a...</t>
+          <t>...Banksy, have achieved international fame despite remaining anonymous. Today, many cities actively encourage street art (12) by designating legal walls where artists can work freely. Today, street art has gained recognition and,...</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>...art (12) by designating legal walls where artists can work freely. Today, street art has gained recognition and, (13) as a result, vibrant neighbourhoods dedicated to this art form have emerged worldwide. Street art festivals are held...</t>
+          <t>...by designating legal walls where artists can work freely. Today, street art has gained recognition and, (13) as a result, vibrant neighbourhoods dedicated to this art form have emerged worldwide. Street art festivals are held...</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
@@ -1507,12 +1509,12 @@
       </c>
       <c r="H9" s="3" t="inlineStr">
         <is>
-          <t>...to collaborate and share their work. Critics argue that street art should remain rebellious and anti-establishment, (15) while supporters believe that recognition helps artists earn a living. Whatever your view, there's no denying (16)...</t>
+          <t>...to collaborate and share their work. Critics argue that street art should remain rebellious and anti-establishment, (15) while supporters believe that recognition helps artists earn a living. Whatever your view, there's no denying...</t>
         </is>
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>...(15) while supporters believe that recognition helps artists earn a living. Whatever your view, there's no denying (16) that street art has become an integral part of contemporary urban culture.</t>
+          <t>...while supporters believe that recognition helps artists earn a living. Whatever your view, there's no denying (16) that street art has become an integral part of contemporary urban culture.</t>
         </is>
       </c>
       <c r="J9" s="3" t="inlineStr">
@@ -1596,28 +1598,28 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="60" customHeight="1">
+    <row r="10">
       <c r="A10" s="2" t="n">
         <v>9</v>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>...sleep to understand why we need it and what happens when we don't get sufficient rest. During sleep, our brains go (9) through different stages, each serving a specific purpose. The deepest stage, known (10) as REM sleep, is when most...</t>
+          <t>...sleep to understand why we need it and what happens when we don't get sufficient rest. During sleep, our brains go (9) through different stages, each serving a specific purpose. The deepest stage, known...</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>...During sleep, our brains go (9) through different stages, each serving a specific purpose. The deepest stage, known (10) as REM sleep, is when most dreaming occurs and plays a crucial role (11) in memory consolidation and learning....</t>
+          <t>...through different stages, each serving a specific purpose. The deepest stage, known (10) as REM sleep, is when most dreaming occurs and plays a crucial role...</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>...a specific purpose. The deepest stage, known (10) as REM sleep, is when most dreaming occurs and plays a crucial role (11) in memory consolidation and learning. Research has shown that people (12) who don't get enough sleep have difficulty...</t>
+          <t>...as REM sleep, is when most dreaming occurs and plays a crucial role (11) in memory consolidation and learning. Research has shown that people...</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>...dreaming occurs and plays a crucial role (11) in memory consolidation and learning. Research has shown that people (12) who don't get enough sleep have difficulty concentrating and are more likely to make mistakes at work or school. Lack...</t>
+          <t>...in memory consolidation and learning. Research has shown that people (12) who don't get enough sleep have difficulty concentrating and are more likely to make mistakes at work or school. Lack...</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -1632,12 +1634,12 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>...recommended seven to nine hours per night. Experts suggest establishing a regular sleep schedule and avoiding screens (15) before bedtime to improve sleep quality. Creating (16) a dark, quiet, and cool bedroom environment can also help...</t>
+          <t>...recommended seven to nine hours per night. Experts suggest establishing a regular sleep schedule and avoiding screens (15) before bedtime to improve sleep quality. Creating...</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>...establishing a regular sleep schedule and avoiding screens (15) before bedtime to improve sleep quality. Creating (16) a dark, quiet, and cool bedroom environment can also help promote better rest and ensure you wake up feeling refreshed.</t>
+          <t>...before bedtime to improve sleep quality. Creating (16) a dark, quiet, and cool bedroom environment can also help promote better rest and ensure you wake up feeling refreshed.</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
@@ -1721,28 +1723,28 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="60" customHeight="1">
+    <row r="11">
       <c r="A11" s="3" t="n">
         <v>10</v>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>...years, it served as the main conduit for commerce, culture, and ideas between Asia and Europe. The route got its name (9) from the lucrative silk trade that originated in China, although many other goods (10) were also transported along...</t>
+          <t>...years, it served as the main conduit for commerce, culture, and ideas between Asia and Europe. The route got its name (9) from the lucrative silk trade that originated in China, although many other goods...</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>...Europe. The route got its name (9) from the lucrative silk trade that originated in China, although many other goods (10) were also transported along these paths, including spices, precious metals, and gemstones. Merchants would travel for...</t>
+          <t>...from the lucrative silk trade that originated in China, although many other goods (10) were also transported along these paths, including spices, precious metals, and gemstones. Merchants would travel for...</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>...including spices, precious metals, and gemstones. Merchants would travel for months, crossing deserts and mountains, (11) to reach distant markets. The Silk Road (12) was not only important for trade but also played a crucial role in...</t>
+          <t>...including spices, precious metals, and gemstones. Merchants would travel for months, crossing deserts and mountains, (11) to reach distant markets. The Silk Road...</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>...Merchants would travel for months, crossing deserts and mountains, (11) to reach distant markets. The Silk Road (12) was not only important for trade but also played a crucial role in spreading religions, technologies, and artistic...</t>
+          <t>...to reach distant markets. The Silk Road (12) was not only important for trade but also played a crucial role in spreading religions, technologies, and artistic...</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
@@ -1752,12 +1754,12 @@
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>...cultural centres where different civilizations met and exchanged ideas. However, the Silk Road's importance declined (14) after the 15th century when maritime routes were developed. Despite this, its legacy (15) has endured, shaping the...</t>
+          <t>...cultural centres where different civilizations met and exchanged ideas. However, the Silk Road's importance declined (14) after the 15th century when maritime routes were developed. Despite this, its legacy...</t>
         </is>
       </c>
       <c r="H11" s="3" t="inlineStr">
         <is>
-          <t>...Road's importance declined (14) after the 15th century when maritime routes were developed. Despite this, its legacy (15) has endured, shaping the development of many societies. Today, historians continue to study the Silk Road to better...</t>
+          <t>...after the 15th century when maritime routes were developed. Despite this, its legacy (15) has endured, shaping the development of many societies. Today, historians continue to study the Silk Road to better...</t>
         </is>
       </c>
       <c r="I11" s="3" t="inlineStr">
@@ -1846,7 +1848,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="60" customHeight="1">
+    <row r="12">
       <c r="A12" s="2" t="n">
         <v>11</v>
       </c>
@@ -1867,27 +1869,27 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>...comes from and the importance of caring for the environment. Many cities now recognise the value of these spaces and (12) are taking steps to support them through grants and land allocation. Some urban gardens focus (13) on growing...</t>
+          <t>...comes from and the importance of caring for the environment. Many cities now recognise the value of these spaces and (12) are taking steps to support them through grants and land allocation. Some urban gardens focus...</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>...of these spaces and (12) are taking steps to support them through grants and land allocation. Some urban gardens focus (13) on growing vegetables and herbs, while others cultivate flowers to attract pollinators like bees and butterflies....</t>
+          <t>...are taking steps to support them through grants and land allocation. Some urban gardens focus (13) on growing vegetables and herbs, while others cultivate flowers to attract pollinators like bees and butterflies....</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>...others cultivate flowers to attract pollinators like bees and butterflies. Despite limited space, creative solutions (14) such as vertical gardens and container planting allow city dwellers to maximise their growing potential. (15) Whether...</t>
+          <t>...others cultivate flowers to attract pollinators like bees and butterflies. Despite limited space, creative solutions (14) such as vertical gardens and container planting allow city dwellers to maximise their growing potential....</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>...(14) such as vertical gardens and container planting allow city dwellers to maximise their growing potential. (15) Whether you have a small windowsill or a large plot, urban gardening offers (16) an accessible way to contribute to a...</t>
+          <t>...such as vertical gardens and container planting allow city dwellers to maximise their growing potential. (15) Whether you have a small windowsill or a large plot, urban gardening offers...</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>...to maximise their growing potential. (15) Whether you have a small windowsill or a large plot, urban gardening offers (16) an accessible way to contribute to a greener, more sustainable urban environment.</t>
+          <t>...Whether you have a small windowsill or a large plot, urban gardening offers (16) an accessible way to contribute to a greener, more sustainable urban environment.</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
@@ -1971,28 +1973,28 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="60" customHeight="1">
+    <row r="13">
       <c r="A13" s="3" t="n">
         <v>12</v>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>...as solar, wind, and hydroelectric power produce little or no greenhouse gas emissions. Solar power harnesses energy (9) from the sun using photovoltaic panels that convert sunlight into electricity. Wind turbines, (10) which can be...</t>
+          <t>...as solar, wind, and hydroelectric power produce little or no greenhouse gas emissions. Solar power harnesses energy (9) from the sun using photovoltaic panels that convert sunlight into electricity. Wind turbines,...</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>...harnesses energy (9) from the sun using photovoltaic panels that convert sunlight into electricity. Wind turbines, (10) which can be installed both on land and offshore, capture the kinetic energy of moving air. These technologies have...</t>
+          <t>...from the sun using photovoltaic panels that convert sunlight into electricity. Wind turbines, (10) which can be installed both on land and offshore, capture the kinetic energy of moving air. These technologies have...</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>...both on land and offshore, capture the kinetic energy of moving air. These technologies have improved dramatically (11) over the past few decades, becoming more efficient and affordable. Many countries (12) have set ambitious targets to...</t>
+          <t>...both on land and offshore, capture the kinetic energy of moving air. These technologies have improved dramatically (11) over the past few decades, becoming more efficient and affordable. Many countries...</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>...have improved dramatically (11) over the past few decades, becoming more efficient and affordable. Many countries (12) have set ambitious targets to increase their use of renewable energy in the coming years. However, renewable energy...</t>
+          <t>...over the past few decades, becoming more efficient and affordable. Many countries (12) have set ambitious targets to increase their use of renewable energy in the coming years. However, renewable energy...</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
@@ -2007,12 +2009,12 @@
       </c>
       <c r="H13" s="3" t="inlineStr">
         <is>
-          <t>...to address this issue. Despite these obstacles, renewable energy capacity continues to grow rapidly around the world. (15) If current trends continue, renewables could/may/might provide the majority of the world's electricity (16) by the...</t>
+          <t>...to address this issue. Despite these obstacles, renewable energy capacity continues to grow rapidly around the world. (15) If current trends continue, renewables could/may/might provide the majority of the world's electricity...</t>
         </is>
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>...the world. (15) If current trends continue, renewables could/may/might provide the majority of the world's electricity (16) by the middle of this century, helping to combat climate change.</t>
+          <t>...If current trends continue, renewables could/may/might provide the majority of the world's electricity (16) by the middle of this century, helping to combat climate change.</t>
         </is>
       </c>
       <c r="J13" s="3" t="inlineStr">
@@ -2096,28 +2098,28 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="60" customHeight="1">
+    <row r="14">
       <c r="A14" s="2" t="n">
         <v>13</v>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>...concerned about its impact on mental health, particularly among young people. Studies have found a correlation (9) between heavy social media use and increased rates of anxiety and depression. One reason for this may/might/could (10)...</t>
+          <t>...concerned about its impact on mental health, particularly among young people. Studies have found a correlation (9) between heavy social media use and increased rates of anxiety and depression. One reason for this may/might/could...</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>...(9) between heavy social media use and increased rates of anxiety and depression. One reason for this may/might/could (10) be that people constantly compare themselves to others' carefully curated online personas, (11) which can lead to...</t>
+          <t>...between heavy social media use and increased rates of anxiety and depression. One reason for this may/might/could (10) be that people constantly compare themselves to others' carefully curated online personas,...</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>...this may/might/could (10) be that people constantly compare themselves to others' carefully curated online personas, (11) which can lead to feelings of inadequacy. The pressure to receive likes and comments is (12) such that a culture has...</t>
+          <t>...be that people constantly compare themselves to others' carefully curated online personas, (11) which can lead to feelings of inadequacy. The pressure to receive likes and comments is...</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>...curated online personas, (11) which can lead to feelings of inadequacy. The pressure to receive likes and comments is (12) such that a culture has formed in which self-worth is often measured by online validation. However, social media is...</t>
+          <t>...which can lead to feelings of inadequacy. The pressure to receive likes and comments is (12) such that a culture has formed in which self-worth is often measured by online validation. However, social media is...</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
@@ -2132,12 +2134,12 @@
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>...for raising awareness about important social issues. Experts recommend limiting screen time and being mindful (15) of how social media makes you feel. (16) If you notice it affecting your mood negatively, it may be time to take a...</t>
+          <t>...for raising awareness about important social issues. Experts recommend limiting screen time and being mindful (15) of how social media makes you feel....</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>...social issues. Experts recommend limiting screen time and being mindful (15) of how social media makes you feel. (16) If you notice it affecting your mood negatively, it may be time to take a break and focus on real-world connections.</t>
+          <t>...of how social media makes you feel. (16) If you notice it affecting your mood negatively, it may be time to take a break and focus on real-world connections.</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
@@ -2221,7 +2223,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="60" customHeight="1">
+    <row r="15">
       <c r="A15" s="3" t="n">
         <v>14</v>
       </c>
@@ -2237,32 +2239,32 @@
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>...a splash. This biomimetic design reduced noise and increased the train's speed. Another fascinating example is Velcro, (11) which was invented after a Swiss engineer noticed how burrs stuck to his dog's fur. The lotus leaf (12) has inspired...</t>
+          <t>...a splash. This biomimetic design reduced noise and increased the train's speed. Another fascinating example is Velcro, (11) which was invented after a Swiss engineer noticed how burrs stuck to his dog's fur. The lotus leaf...</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>...is Velcro, (11) which was invented after a Swiss engineer noticed how burrs stuck to his dog's fur. The lotus leaf (12) has inspired self-cleaning surfaces because water droplets pick up dirt as they roll (13) off the leaf's waxy surface....</t>
+          <t>...which was invented after a Swiss engineer noticed how burrs stuck to his dog's fur. The lotus leaf (12) has inspired self-cleaning surfaces because water droplets pick up dirt as they roll...</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>...dog's fur. The lotus leaf (12) has inspired self-cleaning surfaces because water droplets pick up dirt as they roll (13) off the leaf's waxy surface. Shark skin has influenced swimsuit design, (14) while termite mounds have provided...</t>
+          <t>...has inspired self-cleaning surfaces because water droplets pick up dirt as they roll (13) off the leaf's waxy surface. Shark skin has influenced swimsuit design,...</t>
         </is>
       </c>
       <c r="G15" s="3" t="inlineStr">
         <is>
-          <t>...water droplets pick up dirt as they roll (13) off the leaf's waxy surface. Shark skin has influenced swimsuit design, (14) while termite mounds have provided insights into building ventilation systems that don't require air conditioning. As...</t>
+          <t>...off the leaf's waxy surface. Shark skin has influenced swimsuit design, (14) while termite mounds have provided insights into building ventilation systems that don't require air conditioning. As...</t>
         </is>
       </c>
       <c r="H15" s="3" t="inlineStr">
         <is>
-          <t>...ventilation systems that don't require air conditioning. As we face environmental challenges, biomimicry offers (15) a promising approach to developing sustainable solutions. (16) By learning from nature's time-tested patterns, we can...</t>
+          <t>...ventilation systems that don't require air conditioning. As we face environmental challenges, biomimicry offers (15) a promising approach to developing sustainable solutions....</t>
         </is>
       </c>
       <c r="I15" s="3" t="inlineStr">
         <is>
-          <t>...As we face environmental challenges, biomimicry offers (15) a promising approach to developing sustainable solutions. (16) By learning from nature's time-tested patterns, we can create technologies that work with natural systems rather than...</t>
+          <t>...a promising approach to developing sustainable solutions. (16) By learning from nature's time-tested patterns, we can create technologies that work with natural systems rather than...</t>
         </is>
       </c>
       <c r="J15" s="3" t="inlineStr">
@@ -2346,7 +2348,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="60" customHeight="1">
+    <row r="16">
       <c r="A16" s="2" t="n">
         <v>15</v>
       </c>
@@ -2357,32 +2359,32 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>...ancient India, where a game called Chaturanga was played in the 6th century. From India, the game spread to Persia and (10) then to the Islamic world. (11) When the Moors invaded Spain in the 8th century, they brought chess with them, and it...</t>
+          <t>...ancient India, where a game called Chaturanga was played in the 6th century. From India, the game spread to Persia and (10) then to the Islamic world....</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>...Chaturanga was played in the 6th century. From India, the game spread to Persia and (10) then to the Islamic world. (11) When the Moors invaded Spain in the 8th century, they brought chess with them, and it gradually became popular...</t>
+          <t>...then to the Islamic world. (11) When the Moors invaded Spain in the 8th century, they brought chess with them, and it gradually became popular...</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>...the 8th century, they brought chess with them, and it gradually became popular throughout Europe. The rules of chess (12) have evolved significantly over the centuries. The modern version of the game, (13) which we play today, was...</t>
+          <t>...the 8th century, they brought chess with them, and it gradually became popular throughout Europe. The rules of chess (12) have evolved significantly over the centuries. The modern version of the game,...</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>...Europe. The rules of chess (12) have evolved significantly over the centuries. The modern version of the game, (13) which we play today, was standardised in the 19th century. Chess requires players to think several moves ahead and...</t>
+          <t>...have evolved significantly over the centuries. The modern version of the game, (13) which we play today, was standardised in the 19th century. Chess requires players to think several moves ahead and...</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>...in the 19th century. Chess requires players to think several moves ahead and consider multiple strategies, (14) making it an excellent tool for developing critical thinking and problem-solving skills. The game has (15) also been...</t>
+          <t>...in the 19th century. Chess requires players to think several moves ahead and consider multiple strategies, (14) making it an excellent tool for developing critical thinking and problem-solving skills. The game has...</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>...strategies, (14) making it an excellent tool for developing critical thinking and problem-solving skills. The game has (15) also been studied extensively by psychologists and computer scientists interested in artificial intelligence. Today,...</t>
+          <t>...making it an excellent tool for developing critical thinking and problem-solving skills. The game has (15) also been studied extensively by psychologists and computer scientists interested in artificial intelligence. Today,...</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
@@ -2471,43 +2473,43 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="60" customHeight="1">
+    <row r="17">
       <c r="A17" s="3" t="n">
         <v>16</v>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>...occurs when corals expel the colourful algae living in their tissues, turning completely white. Corals and algae have (9) a symbiotic relationship, meaning they both benefit from living together. The algae provide the coral (10) with food...</t>
+          <t>...occurs when corals expel the colourful algae living in their tissues, turning completely white. Corals and algae have (9) a symbiotic relationship, meaning they both benefit from living together. The algae provide the coral...</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>...algae have (9) a symbiotic relationship, meaning they both benefit from living together. The algae provide the coral (10) with food through photosynthesis, while the coral offers the algae a protected environment. However, (11) when ocean...</t>
+          <t>...a symbiotic relationship, meaning they both benefit from living together. The algae provide the coral (10) with food through photosynthesis, while the coral offers the algae a protected environment. However,...</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>...the coral (10) with food through photosynthesis, while the coral offers the algae a protected environment. However, (11) when ocean temperatures rise even by just one or two degrees, corals become stressed and expel the algae. Without...</t>
+          <t>...with food through photosynthesis, while the coral offers the algae a protected environment. However, (11) when ocean temperatures rise even by just one or two degrees, corals become stressed and expel the algae. Without...</t>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>...their algae, corals lose their main food source and their vibrant colours. Bleached corals are not dead, but they (12) are much more vulnerable to disease and death. (13) If conditions improve quickly, corals can sometimes recover....</t>
+          <t>...their algae, corals lose their main food source and their vibrant colours. Bleached corals are not dead, but they (12) are much more vulnerable to disease and death....</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>...and their vibrant colours. Bleached corals are not dead, but they (12) are much more vulnerable to disease and death. (13) If conditions improve quickly, corals can sometimes recover. Unfortunately, mass bleaching events (14) have become...</t>
+          <t>...are much more vulnerable to disease and death. (13) If conditions improve quickly, corals can sometimes recover. Unfortunately, mass bleaching events...</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
         <is>
-          <t>...and death. (13) If conditions improve quickly, corals can sometimes recover. Unfortunately, mass bleaching events (14) have become more frequent in recent years due to rising ocean temperatures. The Great Barrier Reef (15) has...</t>
+          <t>...If conditions improve quickly, corals can sometimes recover. Unfortunately, mass bleaching events (14) have become more frequent in recent years due to rising ocean temperatures. The Great Barrier Reef...</t>
         </is>
       </c>
       <c r="H17" s="3" t="inlineStr">
         <is>
-          <t>...events (14) have become more frequent in recent years due to rising ocean temperatures. The Great Barrier Reef (15) has experienced several major bleaching events since 2016, with devastating consequences for marine life. Scientists...</t>
+          <t>...have become more frequent in recent years due to rising ocean temperatures. The Great Barrier Reef (15) has experienced several major bleaching events since 2016, with devastating consequences for marine life. Scientists...</t>
         </is>
       </c>
       <c r="I17" s="3" t="inlineStr">
@@ -2596,7 +2598,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="60" customHeight="1">
+    <row r="18">
       <c r="A18" s="2" t="n">
         <v>17</v>
       </c>
@@ -2622,22 +2624,22 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>...It appears that birds use multiple methods, including the sun, stars, and Earth's magnetic field. Some species (13) can even detect polarised light, which helps them orient themselves. Young birds often make their first migration (14)...</t>
+          <t>...It appears that birds use multiple methods, including the sun, stars, and Earth's magnetic field. Some species (13) can even detect polarised light, which helps them orient themselves. Young birds often make their first migration...</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>...(13) can even detect polarised light, which helps them orient themselves. Young birds often make their first migration (14) without their parents, relying entirely on instinct. Climate change is affecting migration patterns, (15) with some...</t>
+          <t>...can even detect polarised light, which helps them orient themselves. Young birds often make their first migration (14) without their parents, relying entirely on instinct. Climate change is affecting migration patterns,...</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>...migration (14) without their parents, relying entirely on instinct. Climate change is affecting migration patterns, (15) with some species arriving at their destinations earlier each year. Habitat loss along migration routes (16) has also...</t>
+          <t>...without their parents, relying entirely on instinct. Climate change is affecting migration patterns, (15) with some species arriving at their destinations earlier each year. Habitat loss along migration routes...</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>...patterns, (15) with some species arriving at their destinations earlier each year. Habitat loss along migration routes (16) has also made these journeys more dangerous, as birds struggle to find suitable places to rest and refuel.</t>
+          <t>...with some species arriving at their destinations earlier each year. Habitat loss along migration routes (16) has also made these journeys more dangerous, as birds struggle to find suitable places to rest and refuel.</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
@@ -2721,7 +2723,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="60" customHeight="1">
+    <row r="19">
       <c r="A19" s="3" t="n">
         <v>18</v>
       </c>
@@ -2732,12 +2734,12 @@
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>...harsh conditions found at great depths. The pressure increases dramatically as you descend, and temperatures can drop (10) to near freezing. There is no sunlight below 1,000 metres, (11) which means that plants cannot grow and creatures must...</t>
+          <t>...harsh conditions found at great depths. The pressure increases dramatically as you descend, and temperatures can drop (10) to near freezing. There is no sunlight below 1,000 metres,...</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>...dramatically as you descend, and temperatures can drop (10) to near freezing. There is no sunlight below 1,000 metres, (11) which means that plants cannot grow and creatures must find other sources of food. Despite these challenges,...</t>
+          <t>...to near freezing. There is no sunlight below 1,000 metres, (11) which means that plants cannot grow and creatures must find other sources of food. Despite these challenges,...</t>
         </is>
       </c>
       <c r="E19" s="3" t="inlineStr">
@@ -2747,17 +2749,17 @@
       </c>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>...like giant squid, anglerfish, and tube worms thrive in this dark world. Many deep-sea animals produce their own light (13) through bioluminescence, using it to attract prey or communicate. Hydrothermal vents, (14) where superheated water...</t>
+          <t>...like giant squid, anglerfish, and tube worms thrive in this dark world. Many deep-sea animals produce their own light (13) through bioluminescence, using it to attract prey or communicate. Hydrothermal vents,...</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
         <is>
-          <t>...produce their own light (13) through bioluminescence, using it to attract prey or communicate. Hydrothermal vents, (14) where superheated water emerges from the ocean floor, support entire ecosystems based on chemical energy rather (15)...</t>
+          <t>...through bioluminescence, using it to attract prey or communicate. Hydrothermal vents, (14) where superheated water emerges from the ocean floor, support entire ecosystems based on chemical energy rather...</t>
         </is>
       </c>
       <c r="H19" s="3" t="inlineStr">
         <is>
-          <t>...(14) where superheated water emerges from the ocean floor, support entire ecosystems based on chemical energy rather (15) than sunlight. Modern technology, including remotely operated vehicles and advanced sonar systems, allows researchers...</t>
+          <t>...where superheated water emerges from the ocean floor, support entire ecosystems based on chemical energy rather (15) than sunlight. Modern technology, including remotely operated vehicles and advanced sonar systems, allows researchers...</t>
         </is>
       </c>
       <c r="I19" s="3" t="inlineStr">
@@ -2846,7 +2848,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="60" customHeight="1">
+    <row r="20">
       <c r="A20" s="2" t="n">
         <v>19</v>
       </c>
@@ -2862,17 +2864,17 @@
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>...communities, providing benefits to both parties. Volunteers gain valuable life experience and cultural understanding, (11) while host communities receive much-needed support and resources. However, critics raise concerns (12) about the...</t>
+          <t>...communities, providing benefits to both parties. Volunteers gain valuable life experience and cultural understanding, (11) while host communities receive much-needed support and resources. However, critics raise concerns...</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>...understanding, (11) while host communities receive much-needed support and resources. However, critics raise concerns (12) about the effectiveness and ethics of short-term volunteer projects. They argue that volunteers often find (13)...</t>
+          <t>...while host communities receive much-needed support and resources. However, critics raise concerns (12) about the effectiveness and ethics of short-term volunteer projects. They argue that volunteers often find...</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>...(12) about the effectiveness and ethics of short-term volunteer projects. They argue that volunteers often find (13) themselves unable to make a real difference due to insufficient training. In some cases, projects may be designed more...</t>
+          <t>...about the effectiveness and ethics of short-term volunteer projects. They argue that volunteers often find (13) themselves unable to make a real difference due to insufficient training. In some cases, projects may be designed more...</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -2882,12 +2884,12 @@
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>...instances where poorly planned voluntourism has actually caused harm to communities or wildlife. Experts recommend (15) that anyone considering volunteer tourism should research organisations carefully. Look for programmes that work (16)...</t>
+          <t>...instances where poorly planned voluntourism has actually caused harm to communities or wildlife. Experts recommend (15) that anyone considering volunteer tourism should research organisations carefully. Look for programmes that work...</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>...(15) that anyone considering volunteer tourism should research organisations carefully. Look for programmes that work (16) in close partnership with local communities and maintain a long-term commitment to sustainable development. The goal...</t>
+          <t>...that anyone considering volunteer tourism should research organisations carefully. Look for programmes that work (16) in close partnership with local communities and maintain a long-term commitment to sustainable development. The goal...</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
@@ -2971,7 +2973,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="60" customHeight="1">
+    <row r="21">
       <c r="A21" s="3" t="n">
         <v>20</v>
       </c>
@@ -3096,7 +3098,7 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="60" customHeight="1">
+    <row r="22">
       <c r="A22" s="2" t="n">
         <v>21</v>
       </c>
@@ -3122,12 +3124,12 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>...it produces methane, a greenhouse gas that is far more potent than carbon dioxide. Additionally, all the resources (13) used to produce that wasted food – including water, energy, and land – are also wasted. If food waste (14) were a...</t>
+          <t>...it produces methane, a greenhouse gas that is far more potent than carbon dioxide. Additionally, all the resources (13) used to produce that wasted food – including water, energy, and land – are also wasted. If food waste...</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>...resources (13) used to produce that wasted food – including water, energy, and land – are also wasted. If food waste (14) were a country, it would be the third largest emitter of greenhouse gases after the United States and China....</t>
+          <t>...used to produce that wasted food – including water, energy, and land – are also wasted. If food waste (14) were a country, it would be the third largest emitter of greenhouse gases after the United States and China....</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
@@ -3221,7 +3223,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="60" customHeight="1">
+    <row r="23">
       <c r="A23" s="3" t="n">
         <v>22</v>
       </c>
@@ -3237,12 +3239,12 @@
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>...analysed to help city planners make better decisions. For example, smart traffic lights can adjust their timing based (11) on real-time traffic flow, reducing congestion and emissions. Many cities have installed smart energy grids (12) that...</t>
+          <t>...analysed to help city planners make better decisions. For example, smart traffic lights can adjust their timing based (11) on real-time traffic flow, reducing congestion and emissions. Many cities have installed smart energy grids...</t>
         </is>
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>...based (11) on real-time traffic flow, reducing congestion and emissions. Many cities have installed smart energy grids (12) that can balance electricity supply and demand more effectively. Smart waste management systems use sensors in bins to...</t>
+          <t>...on real-time traffic flow, reducing congestion and emissions. Many cities have installed smart energy grids (12) that can balance electricity supply and demand more effectively. Smart waste management systems use sensors in bins to...</t>
         </is>
       </c>
       <c r="F23" s="3" t="inlineStr">
@@ -3252,12 +3254,12 @@
       </c>
       <c r="G23" s="3" t="inlineStr">
         <is>
-          <t>...more efficiently. However, smart cities face challenges. The technology requires significant investment, and there (14) are concerns about data privacy and security. Critics worry that not all residents are able (15) to benefit equally...</t>
+          <t>...more efficiently. However, smart cities face challenges. The technology requires significant investment, and there (14) are concerns about data privacy and security. Critics worry that not all residents are able...</t>
         </is>
       </c>
       <c r="H23" s="3" t="inlineStr">
         <is>
-          <t>...investment, and there (14) are concerns about data privacy and security. Critics worry that not all residents are able (15) to benefit equally from these innovations, potentially creating a digital divide. Despite these issues, the smart city...</t>
+          <t>...are concerns about data privacy and security. Critics worry that not all residents are able (15) to benefit equally from these innovations, potentially creating a digital divide. Despite these issues, the smart city...</t>
         </is>
       </c>
       <c r="I23" s="3" t="inlineStr">
@@ -3346,33 +3348,33 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="60" customHeight="1">
+    <row r="24">
       <c r="A24" s="2" t="n">
         <v>23</v>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>...development that transformed communication and the spread of knowledge. The credit for inventing paper goes (9) to Cai Lun, a Chinese court official who developed the process around 105 CE. Before paper, the Chinese wrote (10) on...</t>
+          <t>...development that transformed communication and the spread of knowledge. The credit for inventing paper goes (9) to Cai Lun, a Chinese court official who developed the process around 105 CE. Before paper, the Chinese wrote...</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>...goes (9) to Cai Lun, a Chinese court official who developed the process around 105 CE. Before paper, the Chinese wrote (10) on bamboo strips and silk, which were either too heavy or too expensive for widespread use. Cai Lun's paper was made...</t>
+          <t>...to Cai Lun, a Chinese court official who developed the process around 105 CE. Before paper, the Chinese wrote (10) on bamboo strips and silk, which were either too heavy or too expensive for widespread use. Cai Lun's paper was made...</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>...or too expensive for widespread use. Cai Lun's paper was made from tree bark, hemp, and old fishing nets, creating (11) a lightweight and affordable writing material. The knowledge of papermaking spread slowly (12) along the Silk Road. It...</t>
+          <t>...or too expensive for widespread use. Cai Lun's paper was made from tree bark, hemp, and old fishing nets, creating (11) a lightweight and affordable writing material. The knowledge of papermaking spread slowly...</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>...fishing nets, creating (11) a lightweight and affordable writing material. The knowledge of papermaking spread slowly (12) along the Silk Road. It reached the Islamic world by the 8th century, (13) where the technique was refined and paper...</t>
+          <t>...a lightweight and affordable writing material. The knowledge of papermaking spread slowly (12) along the Silk Road. It reached the Islamic world by the 8th century,...</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>...The knowledge of papermaking spread slowly (12) along the Silk Road. It reached the Islamic world by the 8th century, (13) where the technique was refined and paper mills were established. Muslims introduced paper to Europe during their...</t>
+          <t>...along the Silk Road. It reached the Islamic world by the 8th century, (13) where the technique was refined and paper mills were established. Muslims introduced paper to Europe during their...</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -3471,7 +3473,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="60" customHeight="1">
+    <row r="25">
       <c r="A25" s="3" t="n">
         <v>24</v>
       </c>
@@ -3482,17 +3484,17 @@
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>...with city centres sometimes being up to 7 degrees Celsius warmer than nearby countryside. Several factors contribute (10) to this temperature difference. Dark surfaces like asphalt and concrete absorb solar radiation rather (11) than...</t>
+          <t>...with city centres sometimes being up to 7 degrees Celsius warmer than nearby countryside. Several factors contribute (10) to this temperature difference. Dark surfaces like asphalt and concrete absorb solar radiation rather...</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>...contribute (10) to this temperature difference. Dark surfaces like asphalt and concrete absorb solar radiation rather (11) than reflecting it. Additionally, cities have less vegetation, which means (12) there is less cooling through...</t>
+          <t>...to this temperature difference. Dark surfaces like asphalt and concrete absorb solar radiation rather (11) than reflecting it. Additionally, cities have less vegetation, which means...</t>
         </is>
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t>...concrete absorb solar radiation rather (11) than reflecting it. Additionally, cities have less vegetation, which means (12) there is less cooling through evapotranspiration – the process by which plants release water vapour. Urban heat...</t>
+          <t>...than reflecting it. Additionally, cities have less vegetation, which means (12) there is less cooling through evapotranspiration – the process by which plants release water vapour. Urban heat...</t>
         </is>
       </c>
       <c r="F25" s="3" t="inlineStr">
@@ -3596,38 +3598,38 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="60" customHeight="1">
+    <row r="26">
       <c r="A26" s="2" t="n">
         <v>25</v>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>...now found everywhere, from the deepest ocean trenches to Arctic ice and even in the air we breathe. Microplastics come (9) from various sources. Some are intentionally manufactured as microbeads in cosmetics and cleaning products, (10) while...</t>
+          <t>...now found everywhere, from the deepest ocean trenches to Arctic ice and even in the air we breathe. Microplastics come (9) from various sources. Some are intentionally manufactured as microbeads in cosmetics and cleaning products,...</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>...come (9) from various sources. Some are intentionally manufactured as microbeads in cosmetics and cleaning products, (10) while others result from the breakdown of larger plastic items like bottles and bags. When clothes made (11) of...</t>
+          <t>...from various sources. Some are intentionally manufactured as microbeads in cosmetics and cleaning products, (10) while others result from the breakdown of larger plastic items like bottles and bags. When clothes made...</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>...products, (10) while others result from the breakdown of larger plastic items like bottles and bags. When clothes made (11) of synthetic fibres are washed, they release thousands of plastic microfibres into wastewater systems. The...</t>
+          <t>...while others result from the breakdown of larger plastic items like bottles and bags. When clothes made (11) of synthetic fibres are washed, they release thousands of plastic microfibres into wastewater systems. The...</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>...release thousands of plastic microfibres into wastewater systems. The environmental impact of microplastics is still (12) being studied, but early findings are concerning. Marine animals often mistake microplastics for food, leading (13) to...</t>
+          <t>...release thousands of plastic microfibres into wastewater systems. The environmental impact of microplastics is still (12) being studied, but early findings are concerning. Marine animals often mistake microplastics for food, leading...</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>...(12) being studied, but early findings are concerning. Marine animals often mistake microplastics for food, leading (13) to blocked digestive systems and reduced nutrient absorption. Research has shown that microplastics can (14) also...</t>
+          <t>...being studied, but early findings are concerning. Marine animals often mistake microplastics for food, leading (13) to blocked digestive systems and reduced nutrient absorption. Research has shown that microplastics can...</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>...leading (13) to blocked digestive systems and reduced nutrient absorption. Research has shown that microplastics can (14) also accumulate toxic chemicals, which are then transferred to organisms that ingest them. Humans are exposed to...</t>
+          <t>...to blocked digestive systems and reduced nutrient absorption. Research has shown that microplastics can (14) also accumulate toxic chemicals, which are then transferred to organisms that ingest them. Humans are exposed to...</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
@@ -3721,18 +3723,18 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="60" customHeight="1">
+    <row r="27">
       <c r="A27" s="3" t="n">
         <v>26</v>
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>...trees and used the beans to create a bitter ceremonial drink. The Maya and Aztecs considered chocolate sacred and (9) used it in religious ceremonies and as currency. When Spanish conquistadors arrived in the Americas (10) in the 16th...</t>
+          <t>...trees and used the beans to create a bitter ceremonial drink. The Maya and Aztecs considered chocolate sacred and (9) used it in religious ceremonies and as currency. When Spanish conquistadors arrived in the Americas...</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>...sacred and (9) used it in religious ceremonies and as currency. When Spanish conquistadors arrived in the Americas (10) in the 16th century, they were introduced to chocolate by the Aztec emperor Montezuma. The Spanish transformed the...</t>
+          <t>...used it in religious ceremonies and as currency. When Spanish conquistadors arrived in the Americas (10) in the 16th century, they were introduced to chocolate by the Aztec emperor Montezuma. The Spanish transformed the...</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
@@ -3752,12 +3754,12 @@
       </c>
       <c r="G27" s="3" t="inlineStr">
         <is>
-          <t>...people. In 1847, a British company created the first solid chocolate bar, and milk chocolate was invented shortly (14) after. Today, chocolate is (15) a global industry worth billions of dollars. However, there are concerns about...</t>
+          <t>...people. In 1847, a British company created the first solid chocolate bar, and milk chocolate was invented shortly (14) after. Today, chocolate is...</t>
         </is>
       </c>
       <c r="H27" s="3" t="inlineStr">
         <is>
-          <t>...company created the first solid chocolate bar, and milk chocolate was invented shortly (14) after. Today, chocolate is (15) a global industry worth billions of dollars. However, there are concerns about sustainability and fair labour...</t>
+          <t>...after. Today, chocolate is (15) a global industry worth billions of dollars. However, there are concerns about sustainability and fair labour...</t>
         </is>
       </c>
       <c r="I27" s="3" t="inlineStr">
@@ -3846,7 +3848,7 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="60" customHeight="1">
+    <row r="28">
       <c r="A28" s="2" t="n">
         <v>27</v>
       </c>
@@ -3857,12 +3859,12 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>...galaxies through online platforms, or track pollution levels in their neighbourhoods. The data collected by thousands (10) of volunteers can help scientists tackle research questions that would (11) be impossible to address alone due to the...</t>
+          <t>...galaxies through online platforms, or track pollution levels in their neighbourhoods. The data collected by thousands (10) of volunteers can help scientists tackle research questions that would...</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>...The data collected by thousands (10) of volunteers can help scientists tackle research questions that would (11) be impossible to address alone due to the scale of observation required. One of the most successful citizen science...</t>
+          <t>...of volunteers can help scientists tackle research questions that would (11) be impossible to address alone due to the scale of observation required. One of the most successful citizen science...</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
@@ -3882,12 +3884,12 @@
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>...scientific literacy and feel connected to research. Critics worry about data quality, but studies have shown that (15) when properly designed, citizen science projects can produce reliable results. (16) As technology continues to...</t>
+          <t>...scientific literacy and feel connected to research. Critics worry about data quality, but studies have shown that (15) when properly designed, citizen science projects can produce reliable results....</t>
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>...but studies have shown that (15) when properly designed, citizen science projects can produce reliable results. (16) As technology continues to advance, citizen science will likely play an increasingly important role in scientific...</t>
+          <t>...when properly designed, citizen science projects can produce reliable results. (16) As technology continues to advance, citizen science will likely play an increasingly important role in scientific...</t>
         </is>
       </c>
       <c r="J28" s="2" t="inlineStr">
@@ -3971,7 +3973,7 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="60" customHeight="1">
+    <row r="29">
       <c r="A29" s="3" t="n">
         <v>28</v>
       </c>
@@ -4007,12 +4009,12 @@
       </c>
       <c r="H29" s="3" t="inlineStr">
         <is>
-          <t>...and climate control. Critics argue that until renewable energy becomes cheaper, vertical farming may/might/could (15) not be environmentally sustainable. Despite these concerns, vertical farming is expanding rapidly, (16) with...</t>
+          <t>...and climate control. Critics argue that until renewable energy becomes cheaper, vertical farming may/might/could (15) not be environmentally sustainable. Despite these concerns, vertical farming is expanding rapidly,...</t>
         </is>
       </c>
       <c r="I29" s="3" t="inlineStr">
         <is>
-          <t>...(15) not be environmentally sustainable. Despite these concerns, vertical farming is expanding rapidly, (16) with facilities opening in cities worldwide as technology improves and costs decrease.</t>
+          <t>...not be environmentally sustainable. Despite these concerns, vertical farming is expanding rapidly, (16) with facilities opening in cities worldwide as technology improves and costs decrease.</t>
         </is>
       </c>
       <c r="J29" s="3" t="inlineStr">
@@ -4096,18 +4098,18 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="60" customHeight="1">
+    <row r="30">
       <c r="A30" s="2" t="n">
         <v>29</v>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>...kilometres from Canada and the United States to spend winter in Mexico. What makes this migration extraordinary is (9) that the butterflies making the journey have never been to Mexico before. They are following (10) an identical route...</t>
+          <t>...kilometres from Canada and the United States to spend winter in Mexico. What makes this migration extraordinary is (9) that the butterflies making the journey have never been to Mexico before. They are following...</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>...extraordinary is (9) that the butterflies making the journey have never been to Mexico before. They are following (10) an identical route to the one their great-great-grandparents took, relying entirely on instinct. Scientists still...</t>
+          <t>...that the butterflies making the journey have never been to Mexico before. They are following (10) an identical route to the one their great-great-grandparents took, relying entirely on instinct. Scientists still...</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
@@ -4117,12 +4119,12 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>...though it appears they use a combination of the sun's position and Earth's magnetic field. The journey is perilous, (12) with many butterflies dying along the way due to exhaustion, predators, or bad weather. Those (13) which survive reach...</t>
+          <t>...though it appears they use a combination of the sun's position and Earth's magnetic field. The journey is perilous, (12) with many butterflies dying along the way due to exhaustion, predators, or bad weather. Those...</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>...is perilous, (12) with many butterflies dying along the way due to exhaustion, predators, or bad weather. Those (13) which survive reach the oyamel fir forests in Mexico's mountains, where millions of monarchs cluster together on trees...</t>
+          <t>...with many butterflies dying along the way due to exhaustion, predators, or bad weather. Those (13) which survive reach the oyamel fir forests in Mexico's mountains, where millions of monarchs cluster together on trees...</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
@@ -4202,7 +4204,7 @@
       </c>
       <c r="V30" s="2" t="inlineStr">
         <is>
-          <t>Relative pronoun used to introduce a restrictive relative clause modifying 'Those'.</t>
+          <t>Relative pronoun used to introduce a restrictive relative clause modifying 'Those'. 'Which' is preferred in formal written English for this structure.</t>
         </is>
       </c>
       <c r="W30" s="2" t="inlineStr">
@@ -4221,18 +4223,18 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="60" customHeight="1">
+    <row r="31">
       <c r="A31" s="3" t="n">
         <v>30</v>
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>...in understanding how memories are formed, stored, and retrieved. Memory is not a single entity but rather consists (9) of several different systems. Short-term memory holds information temporarily, usually for no more (10) than 20-30...</t>
+          <t>...in understanding how memories are formed, stored, and retrieved. Memory is not a single entity but rather consists (9) of several different systems. Short-term memory holds information temporarily, usually for no more...</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>...rather consists (9) of several different systems. Short-term memory holds information temporarily, usually for no more (10) than 20-30 seconds, while long-term memory can store information for years or even a lifetime. The process of...</t>
+          <t>...of several different systems. Short-term memory holds information temporarily, usually for no more (10) than 20-30 seconds, while long-term memory can store information for years or even a lifetime. The process of...</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
@@ -4346,7 +4348,7 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="60" customHeight="1">
+    <row r="32">
       <c r="A32" s="2" t="n">
         <v>31</v>
       </c>
@@ -4357,27 +4359,27 @@
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>...that they produce zero direct emissions, making them much cleaner for urban air quality. They are also cheaper to run (10) than traditional vehicles because electricity costs less than petrol, and EVs require less maintenance due (11) to...</t>
+          <t>...that they produce zero direct emissions, making them much cleaner for urban air quality. They are also cheaper to run (10) than traditional vehicles because electricity costs less than petrol, and EVs require less maintenance due...</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>...to run (10) than traditional vehicles because electricity costs less than petrol, and EVs require less maintenance due (11) to having fewer moving parts. Many countries offer incentives such as tax breaks to encourage people to switch to...</t>
+          <t>...than traditional vehicles because electricity costs less than petrol, and EVs require less maintenance due (11) to having fewer moving parts. Many countries offer incentives such as tax breaks to encourage people to switch to...</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>...such as tax breaks to encourage people to switch to electric cars. However, there are still challenges that have (12) yet to be fully resolved. The limited driving range of some EVs compared to petrol cars remains a concern, (13)...</t>
+          <t>...such as tax breaks to encourage people to switch to electric cars. However, there are still challenges that have (12) yet to be fully resolved. The limited driving range of some EVs compared to petrol cars remains a concern,...</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>...have (12) yet to be fully resolved. The limited driving range of some EVs compared to petrol cars remains a concern, (13) although battery technology is improving rapidly. Charging infrastructure also needs to expand – (14) while it's easy...</t>
+          <t>...yet to be fully resolved. The limited driving range of some EVs compared to petrol cars remains a concern, (13) although battery technology is improving rapidly. Charging infrastructure also needs to expand –...</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>...a concern, (13) although battery technology is improving rapidly. Charging infrastructure also needs to expand – (14) while it's easy to charge at home, public charging stations are still not widely available in many areas. The...</t>
+          <t>...although battery technology is improving rapidly. Charging infrastructure also needs to expand – (14) while it's easy to charge at home, public charging stations are still not widely available in many areas. The...</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
@@ -4471,7 +4473,7 @@
         </is>
       </c>
     </row>
-    <row r="33" ht="60" customHeight="1">
+    <row r="33">
       <c r="A33" s="3" t="n">
         <v>32</v>
       </c>
@@ -4482,12 +4484,12 @@
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>...in Egypt, which was established in the 3rd century BCE. It aimed to collect all the world's knowledge and is estimated (10) to have contained hundreds of thousands of scrolls. Sadly, the library was destroyed, and much of its collection (11)...</t>
+          <t>...in Egypt, which was established in the 3rd century BCE. It aimed to collect all the world's knowledge and is estimated (10) to have contained hundreds of thousands of scrolls. Sadly, the library was destroyed, and much of its collection...</t>
         </is>
       </c>
       <c r="D33" s="3" t="inlineStr">
         <is>
-          <t>...(10) to have contained hundreds of thousands of scrolls. Sadly, the library was destroyed, and much of its collection (11) was lost forever, representing an irreplaceable loss to human knowledge. During the Middle Ages, libraries were...</t>
+          <t>...to have contained hundreds of thousands of scrolls. Sadly, the library was destroyed, and much of its collection (11) was lost forever, representing an irreplaceable loss to human knowledge. During the Middle Ages, libraries were...</t>
         </is>
       </c>
       <c r="E33" s="3" t="inlineStr">
@@ -4497,17 +4499,17 @@
       </c>
       <c r="F33" s="3" t="inlineStr">
         <is>
-          <t>...manuscripts by hand. The invention of the printing press in the 15th century revolutionised access to books, making (13) them much more affordable and widely available. Public libraries began to emerge in the 19th century, reflecting (14)...</t>
+          <t>...manuscripts by hand. The invention of the printing press in the 15th century revolutionised access to books, making (13) them much more affordable and widely available. Public libraries began to emerge in the 19th century, reflecting...</t>
         </is>
       </c>
       <c r="G33" s="3" t="inlineStr">
         <is>
-          <t>...(13) them much more affordable and widely available. Public libraries began to emerge in the 19th century, reflecting (14) a belief that knowledge should be accessible to all, not just the wealthy. Today, libraries continue to evolve. (15)...</t>
+          <t>...them much more affordable and widely available. Public libraries began to emerge in the 19th century, reflecting (14) a belief that knowledge should be accessible to all, not just the wealthy. Today, libraries continue to evolve....</t>
         </is>
       </c>
       <c r="H33" s="3" t="inlineStr">
         <is>
-          <t>...(14) a belief that knowledge should be accessible to all, not just the wealthy. Today, libraries continue to evolve. (15) While they still lend books, many now offer digital resources, community spaces, and technology access. Some people...</t>
+          <t>...a belief that knowledge should be accessible to all, not just the wealthy. Today, libraries continue to evolve. (15) While they still lend books, many now offer digital resources, community spaces, and technology access. Some people...</t>
         </is>
       </c>
       <c r="I33" s="3" t="inlineStr">
@@ -4596,7 +4598,7 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="60" customHeight="1">
+    <row r="34">
       <c r="A34" s="2" t="n">
         <v>33</v>
       </c>
@@ -4612,17 +4614,17 @@
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>...were reintroduced to Yellowstone National Park in the 1990s, they controlled deer populations, allowing vegetation (11) to recover. This in turn benefited numerous other species, demonstrating (12) how interconnected ecosystems truly are....</t>
+          <t>...were reintroduced to Yellowstone National Park in the 1990s, they controlled deer populations, allowing vegetation (11) to recover. This in turn benefited numerous other species, demonstrating...</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>...deer populations, allowing vegetation (11) to recover. This in turn benefited numerous other species, demonstrating (12) how interconnected ecosystems truly are. Rewilding projects differ (13) both in scale and scope, from small nature...</t>
+          <t>...to recover. This in turn benefited numerous other species, demonstrating (12) how interconnected ecosystems truly are. Rewilding projects differ...</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>...numerous other species, demonstrating (12) how interconnected ecosystems truly are. Rewilding projects differ (13) both in scale and scope, from small nature reserves to vast wilderness areas. Some focus on reintroducing specific...</t>
+          <t>...how interconnected ecosystems truly are. Rewilding projects differ (13) both in scale and scope, from small nature reserves to vast wilderness areas. Some focus on reintroducing specific...</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
@@ -4721,23 +4723,23 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="60" customHeight="1">
+    <row r="35">
       <c r="A35" s="3" t="n">
         <v>34</v>
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>...a crucial role in regulating Earth's climate and supporting marine ecosystems. Surface currents are driven primarily (9) by wind patterns and the Earth's rotation. The Gulf Stream, for example, carries warm water (10) from the tropical...</t>
+          <t>...a crucial role in regulating Earth's climate and supporting marine ecosystems. Surface currents are driven primarily (9) by wind patterns and the Earth's rotation. The Gulf Stream, for example, carries warm water...</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>...are driven primarily (9) by wind patterns and the Earth's rotation. The Gulf Stream, for example, carries warm water (10) from the tropical Atlantic to northern Europe, making the climate there much milder (11) than it would otherwise be....</t>
+          <t>...by wind patterns and the Earth's rotation. The Gulf Stream, for example, carries warm water (10) from the tropical Atlantic to northern Europe, making the climate there much milder...</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t>...example, carries warm water (10) from the tropical Atlantic to northern Europe, making the climate there much milder (11) than it would otherwise be. Without this current, countries like Britain would have winters similar to those of...</t>
+          <t>...from the tropical Atlantic to northern Europe, making the climate there much milder (11) than it would otherwise be. Without this current, countries like Britain would have winters similar to those of...</t>
         </is>
       </c>
       <c r="E35" s="3" t="inlineStr">
@@ -4747,17 +4749,17 @@
       </c>
       <c r="F35" s="3" t="inlineStr">
         <is>
-          <t>...belt', are driven by differences in water temperature and salinity. Cold, salty water is denser and sinks, creating (13) a circulation pattern that moves water between ocean basins. This deep circulation This deep circulation can take (14)...</t>
+          <t>...belt', are driven by differences in water temperature and salinity. Cold, salty water is denser and sinks, creating (13) a circulation pattern that moves water between ocean basins. This deep circulation This deep circulation can take...</t>
         </is>
       </c>
       <c r="G35" s="3" t="inlineStr">
         <is>
-          <t>...(13) a circulation pattern that moves water between ocean basins. This deep circulation This deep circulation can take (14) the equivalent of several centuries to complete one full circuit. Ocean currents transport nutrients, affecting (15)...</t>
+          <t>...a circulation pattern that moves water between ocean basins. This deep circulation This deep circulation can take (14) the equivalent of several centuries to complete one full circuit. Ocean currents transport nutrients, affecting...</t>
         </is>
       </c>
       <c r="H35" s="3" t="inlineStr">
         <is>
-          <t>...(14) the equivalent of several centuries to complete one full circuit. Ocean currents transport nutrients, affecting (15) where fish populations thrive. They also redistribute heat around the planet, influencing weather patterns and...</t>
+          <t>...the equivalent of several centuries to complete one full circuit. Ocean currents transport nutrients, affecting (15) where fish populations thrive. They also redistribute heat around the planet, influencing weather patterns and...</t>
         </is>
       </c>
       <c r="I35" s="3" t="inlineStr">
@@ -4846,7 +4848,7 @@
         </is>
       </c>
     </row>
-    <row r="36" ht="60" customHeight="1">
+    <row r="36">
       <c r="A36" s="2" t="n">
         <v>35</v>
       </c>
@@ -4857,22 +4859,22 @@
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>...appear to be universal. Red, for instance, tends to increase heart rate and create feelings of excitement or urgency, (10) which is why it's often used in warning signs and sale advertisements. Blue generally has (11) a calming effect and is...</t>
+          <t>...appear to be universal. Red, for instance, tends to increase heart rate and create feelings of excitement or urgency, (10) which is why it's often used in warning signs and sale advertisements. Blue generally has...</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>...excitement or urgency, (10) which is why it's often used in warning signs and sale advertisements. Blue generally has (11) a calming effect and is associated with trust and reliability, making it popular for corporate branding. The food...</t>
+          <t>...which is why it's often used in warning signs and sale advertisements. Blue generally has (11) a calming effect and is associated with trust and reliability, making it popular for corporate branding. The food...</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>...with trust and reliability, making it popular for corporate branding. The food industry carefully considers colour (12) when designing packaging and marketing campaigns. Studies have shown that people perceive foods (13) as tasting...</t>
+          <t>...with trust and reliability, making it popular for corporate branding. The food industry carefully considers colour (12) when designing packaging and marketing campaigns. Studies have shown that people perceive foods...</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>...considers colour (12) when designing packaging and marketing campaigns. Studies have shown that people perceive foods (13) as tasting different depending on their colour, even when the actual flavour is identical. Yellow is often used to...</t>
+          <t>...when designing packaging and marketing campaigns. Studies have shown that people perceive foods (13) as tasting different depending on their colour, even when the actual flavour is identical. Yellow is often used to...</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
@@ -4882,12 +4884,12 @@
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>...blues and greens to promote calm, while gyms might use energising reds and oranges. However, it's important to note (15) that individual responses to colour can vary based on personal experiences and cultural background. (16) While colour...</t>
+          <t>...blues and greens to promote calm, while gyms might use energising reds and oranges. However, it's important to note (15) that individual responses to colour can vary based on personal experiences and cultural background....</t>
         </is>
       </c>
       <c r="I36" s="2" t="inlineStr">
         <is>
-          <t>...to note (15) that individual responses to colour can vary based on personal experiences and cultural background. (16) While colour psychology provides useful guidelines, designers must consider the specific context and audience when...</t>
+          <t>...that individual responses to colour can vary based on personal experiences and cultural background. (16) While colour psychology provides useful guidelines, designers must consider the specific context and audience when...</t>
         </is>
       </c>
       <c r="J36" s="2" t="inlineStr">
@@ -4971,18 +4973,18 @@
         </is>
       </c>
     </row>
-    <row r="37" ht="60" customHeight="1">
+    <row r="37">
       <c r="A37" s="3" t="n">
         <v>36</v>
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>...centres, provide invaluable insights into human civilisation. UNESCO's World Heritage List includes over 1,100 sites (9) from around the world, recognising locations that have 'outstanding universal value'. Sites are selected based (10) on...</t>
+          <t>...centres, provide invaluable insights into human civilisation. UNESCO's World Heritage List includes over 1,100 sites (9) from around the world, recognising locations that have 'outstanding universal value'. Sites are selected based...</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>...(9) from around the world, recognising locations that have 'outstanding universal value'. Sites are selected based (10) on strict criteria, including their uniqueness, authenticity, and integrity. Some famous examples include the Pyramids...</t>
+          <t>...from around the world, recognising locations that have 'outstanding universal value'. Sites are selected based (10) on strict criteria, including their uniqueness, authenticity, and integrity. Some famous examples include the Pyramids...</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
@@ -4992,12 +4994,12 @@
       </c>
       <c r="E37" s="3" t="inlineStr">
         <is>
-          <t>...However, preserving heritage sites presents numerous challenges. Natural disasters, climate change, pollution, and war (12) have all taken their toll on precious monuments. Tourism itself can be a double-edged sword – it provides (13) much...</t>
+          <t>...However, preserving heritage sites presents numerous challenges. Natural disasters, climate change, pollution, and war (12) have all taken their toll on precious monuments. Tourism itself can be a double-edged sword – it provides...</t>
         </is>
       </c>
       <c r="F37" s="3" t="inlineStr">
         <is>
-          <t>...and war (12) have all taken their toll on precious monuments. Tourism itself can be a double-edged sword – it provides (13) much needed funding for conservation, yet excessive visitor numbers can damage fragile structures and disturb local...</t>
+          <t>...have all taken their toll on precious monuments. Tourism itself can be a double-edged sword – it provides (13) much needed funding for conservation, yet excessive visitor numbers can damage fragile structures and disturb local...</t>
         </is>
       </c>
       <c r="G37" s="3" t="inlineStr">
@@ -5007,12 +5009,12 @@
       </c>
       <c r="H37" s="3" t="inlineStr">
         <is>
-          <t>...technology to allow people to experience the site without causing physical damage. Local communities should also (15) be involved in preservation decisions, as they often have deep connections to these places. (16) As our world changes...</t>
+          <t>...technology to allow people to experience the site without causing physical damage. Local communities should also (15) be involved in preservation decisions, as they often have deep connections to these places....</t>
         </is>
       </c>
       <c r="I37" s="3" t="inlineStr">
         <is>
-          <t>...should also (15) be involved in preservation decisions, as they often have deep connections to these places. (16) As our world changes rapidly, protecting cultural heritage sites becomes increasingly important for maintaining links...</t>
+          <t>...be involved in preservation decisions, as they often have deep connections to these places. (16) As our world changes rapidly, protecting cultural heritage sites becomes increasingly important for maintaining links...</t>
         </is>
       </c>
       <c r="J37" s="3" t="inlineStr">
@@ -5096,7 +5098,7 @@
         </is>
       </c>
     </row>
-    <row r="38" ht="60" customHeight="1">
+    <row r="38">
       <c r="A38" s="2" t="n">
         <v>37</v>
       </c>
@@ -5122,12 +5124,12 @@
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>...side effects by targeting treatment more precisely. Researchers are also developing nanosensors that could/might/may (13) detect diseases at much earlier stages than current methods allow. Nanotechnology, (14) which has revolutionised the...</t>
+          <t>...side effects by targeting treatment more precisely. Researchers are also developing nanosensors that could/might/may (13) detect diseases at much earlier stages than current methods allow. Nanotechnology,...</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>...that could/might/may (13) detect diseases at much earlier stages than current methods allow. Nanotechnology, (14) which has revolutionised the electronics industry, makes it possible to produce smaller and more powerful computer...</t>
+          <t>...detect diseases at much earlier stages than current methods allow. Nanotechnology, (14) which has revolutionised the electronics industry, makes it possible to produce smaller and more powerful computer...</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
@@ -5207,7 +5209,7 @@
       </c>
       <c r="W38" s="2" t="inlineStr">
         <is>
-          <t>Relative pronoun used to introduce a non-restrictive relative clause giving additional information about 'Nanotechnology...</t>
+          <t>Relative pronoun used to introduce a non-restrictive relative clause giving additional information about 'Nanotechnology'.</t>
         </is>
       </c>
       <c r="X38" s="2" t="inlineStr">
@@ -5221,7 +5223,7 @@
         </is>
       </c>
     </row>
-    <row r="39" ht="60" customHeight="1">
+    <row r="39">
       <c r="A39" s="3" t="n">
         <v>38</v>
       </c>
@@ -5252,17 +5254,17 @@
       </c>
       <c r="G39" s="3" t="inlineStr">
         <is>
-          <t>...of computer animation in the 1990s transformed the industry completely. Pixar's Toy Story, released in 1995, was (14) the first entirely computer-animated feature film. Digital animation has (15) made it possible to create effects and...</t>
+          <t>...of computer animation in the 1990s transformed the industry completely. Pixar's Toy Story, released in 1995, was (14) the first entirely computer-animated feature film. Digital animation has...</t>
         </is>
       </c>
       <c r="H39" s="3" t="inlineStr">
         <is>
-          <t>...Pixar's Toy Story, released in 1995, was (14) the first entirely computer-animated feature film. Digital animation has (15) made it possible to create effects and visual styles that would have been impossible with traditional techniques. (16)...</t>
+          <t>...the first entirely computer-animated feature film. Digital animation has (15) made it possible to create effects and visual styles that would have been impossible with traditional techniques....</t>
         </is>
       </c>
       <c r="I39" s="3" t="inlineStr">
         <is>
-          <t>...(15) made it possible to create effects and visual styles that would have been impossible with traditional techniques. (16) Despite these technological advances, many animators argue that the fundamental principles of timing, movement, and...</t>
+          <t>...made it possible to create effects and visual styles that would have been impossible with traditional techniques. (16) Despite these technological advances, many animators argue that the fundamental principles of timing, movement, and...</t>
         </is>
       </c>
       <c r="J39" s="3" t="inlineStr">
@@ -5346,7 +5348,7 @@
         </is>
       </c>
     </row>
-    <row r="40" ht="60" customHeight="1">
+    <row r="40">
       <c r="A40" s="2" t="n">
         <v>39</v>
       </c>
@@ -5367,22 +5369,22 @@
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>...even when submerged during high tide. These forests provide crucial environmental services. They protect coastlines (12) from erosion and storm damage by absorbing wave energy. During tsunamis and hurricanes, mangrove forests have (13)...</t>
+          <t>...even when submerged during high tide. These forests provide crucial environmental services. They protect coastlines (12) from erosion and storm damage by absorbing wave energy. During tsunamis and hurricanes, mangrove forests have...</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>...(12) from erosion and storm damage by absorbing wave energy. During tsunamis and hurricanes, mangrove forests have (13) been shown to significantly reduce damage to coastal communities. The tangled root systems create nursery habitats for...</t>
+          <t>...from erosion and storm damage by absorbing wave energy. During tsunamis and hurricanes, mangrove forests have (13) been shown to significantly reduce damage to coastal communities. The tangled root systems create nursery habitats for...</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>...species, supporting both biodiversity and local fishing industries. Mangroves are also powerful carbon sinks, storing (14) more carbon per unit area than most tropical forests. Unfortunately, over half of the world's mangrove forests (15)...</t>
+          <t>...species, supporting both biodiversity and local fishing industries. Mangroves are also powerful carbon sinks, storing (14) more carbon per unit area than most tropical forests. Unfortunately, over half of the world's mangrove forests...</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>...(14) more carbon per unit area than most tropical forests. Unfortunately, over half of the world's mangrove forests (15) have been destroyed in recent decades, cleared for coastal development, aquaculture, and agriculture. Conservation...</t>
+          <t>...more carbon per unit area than most tropical forests. Unfortunately, over half of the world's mangrove forests (15) have been destroyed in recent decades, cleared for coastal development, aquaculture, and agriculture. Conservation...</t>
         </is>
       </c>
       <c r="I40" s="2" t="inlineStr">
@@ -5471,23 +5473,23 @@
         </is>
       </c>
     </row>
-    <row r="41" ht="60" customHeight="1">
+    <row r="41">
       <c r="A41" s="3" t="n">
         <v>40</v>
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>...sites like former concentration camps, battlefields, and disaster zones each year. People visit dark tourism sites (9) for various reasons. Some seek to pay respects to victims, while others want to experience historical events (10)...</t>
+          <t>...sites like former concentration camps, battlefields, and disaster zones each year. People visit dark tourism sites (9) for various reasons. Some seek to pay respects to victims, while others want to experience historical events...</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>...sites (9) for various reasons. Some seek to pay respects to victims, while others want to experience historical events (10) rather than simply reading books or watching films about them. Educational purposes are often cited, (11) as these...</t>
+          <t>...for various reasons. Some seek to pay respects to victims, while others want to experience historical events (10) rather than simply reading books or watching films about them. Educational purposes are often cited,...</t>
         </is>
       </c>
       <c r="D41" s="3" t="inlineStr">
         <is>
-          <t>...events (10) rather than simply reading books or watching films about them. Educational purposes are often cited, (11) as these sites offer powerful lessons about human suffering and resilience. Famous dark tourism destinations include...</t>
+          <t>...rather than simply reading books or watching films about them. Educational purposes are often cited, (11) as these sites offer powerful lessons about human suffering and resilience. Famous dark tourism destinations include...</t>
         </is>
       </c>
       <c r="E41" s="3" t="inlineStr">
@@ -5596,7 +5598,7 @@
         </is>
       </c>
     </row>
-    <row r="42" ht="60" customHeight="1">
+    <row r="42">
       <c r="A42" s="2" t="n">
         <v>41</v>
       </c>
@@ -5617,12 +5619,12 @@
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>...can sustainably increase happiness. Regular exercise, maintaining strong social connections, and practicing gratitude (12) have all been proven to boost well-being. People who invest (13) in experiences rather than material possessions tend...</t>
+          <t>...can sustainably increase happiness. Regular exercise, maintaining strong social connections, and practicing gratitude (12) have all been proven to boost well-being. People who invest...</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>...strong social connections, and practicing gratitude (12) have all been proven to boost well-being. People who invest (13) in experiences rather than material possessions tend to be happier, as do those who help others through volunteering...</t>
+          <t>...have all been proven to boost well-being. People who invest (13) in experiences rather than material possessions tend to be happier, as do those who help others through volunteering...</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
@@ -5717,22 +5719,22 @@
       </c>
       <c r="Y42" s="2" t="inlineStr">
         <is>
-          <t>Part of the correlative expression 'not just... but also', used to emphasise that something includes more than one eleme...</t>
+          <t>Part of the correlative expression 'not just... but also', used to emphasise that something includes more than one element.</t>
         </is>
       </c>
     </row>
-    <row r="43" ht="60" customHeight="1">
+    <row r="43">
       <c r="A43" s="3" t="n">
         <v>42</v>
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>...these labels is essential for making informed dietary choices. In most countries, food manufacturers are required (9) by law to list ingredients in descending order by weight. This means the first ingredient listed is present (10) in...</t>
+          <t>...these labels is essential for making informed dietary choices. In most countries, food manufacturers are required (9) by law to list ingredients in descending order by weight. This means the first ingredient listed is present...</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>...(9) by law to list ingredients in descending order by weight. This means the first ingredient listed is present (10) in the greatest quantity. However, manufacturers sometimes use multiple types of sugar with different names to prevent...</t>
+          <t>...by law to list ingredients in descending order by weight. This means the first ingredient listed is present (10) in the greatest quantity. However, manufacturers sometimes use multiple types of sugar with different names to prevent...</t>
         </is>
       </c>
       <c r="D43" s="3" t="inlineStr">
@@ -5742,12 +5744,12 @@
       </c>
       <c r="E43" s="3" t="inlineStr">
         <is>
-          <t>...Nutritional labels typically show the amount of calories, fat, protein, and carbohydrates per serving. The problem is (12) that serving sizes on labels don't always match what people actually eat. A package that appears small might (13) be...</t>
+          <t>...Nutritional labels typically show the amount of calories, fat, protein, and carbohydrates per serving. The problem is (12) that serving sizes on labels don't always match what people actually eat. A package that appears small might...</t>
         </is>
       </c>
       <c r="F43" s="3" t="inlineStr">
         <is>
-          <t>...is (12) that serving sizes on labels don't always match what people actually eat. A package that appears small might (13) be labelled as containing two or more servings, meaning consumers could accidentally consume far more calories than...</t>
+          <t>...that serving sizes on labels don't always match what people actually eat. A package that appears small might (13) be labelled as containing two or more servings, meaning consumers could accidentally consume far more calories than...</t>
         </is>
       </c>
       <c r="G43" s="3" t="inlineStr">
@@ -5846,7 +5848,7 @@
         </is>
       </c>
     </row>
-    <row r="44" ht="60" customHeight="1">
+    <row r="44">
       <c r="A44" s="2" t="n">
         <v>43</v>
       </c>
@@ -5862,12 +5864,12 @@
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>...like Nikola Tesla and Heinrich Hertz. Marconi successfully demonstrated long-distance wireless communication in 1901, (11) when he transmitted a signal across the Atlantic Ocean. In its early days, radio was primarily used (12) for...</t>
+          <t>...like Nikola Tesla and Heinrich Hertz. Marconi successfully demonstrated long-distance wireless communication in 1901, (11) when he transmitted a signal across the Atlantic Ocean. In its early days, radio was primarily used...</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>...in 1901, (11) when he transmitted a signal across the Atlantic Ocean. In its early days, radio was primarily used (12) for ship-to-shore communication and military purposes. Commercial broadcasting began in the 1920s, and radio quickly...</t>
+          <t>...when he transmitted a signal across the Atlantic Ocean. In its early days, radio was primarily used (12) for ship-to-shore communication and military purposes. Commercial broadcasting began in the 1920s, and radio quickly...</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
@@ -5971,28 +5973,28 @@
         </is>
       </c>
     </row>
-    <row r="45" ht="60" customHeight="1">
+    <row r="45">
       <c r="A45" s="3" t="n">
         <v>44</v>
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>...the importance of bees for pollination and food security. Surprisingly, cities can actually provide excellent habitats (9) for bees. Urban areas often have diverse flowering plants throughout the growing season, from gardens and parks (10)...</t>
+          <t>...the importance of bees for pollination and food security. Surprisingly, cities can actually provide excellent habitats (9) for bees. Urban areas often have diverse flowering plants throughout the growing season, from gardens and parks...</t>
         </is>
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>...(9) for bees. Urban areas often have diverse flowering plants throughout the growing season, from gardens and parks (10) to roadside plantings. Cities also tend to use fewer pesticides than agricultural areas, (11) which can be harmful to...</t>
+          <t>...for bees. Urban areas often have diverse flowering plants throughout the growing season, from gardens and parks (10) to roadside plantings. Cities also tend to use fewer pesticides than agricultural areas,...</t>
         </is>
       </c>
       <c r="D45" s="3" t="inlineStr">
         <is>
-          <t>...from gardens and parks (10) to roadside plantings. Cities also tend to use fewer pesticides than agricultural areas, (11) which can be harmful to bee populations. Urban bees have been found to produce high-quality honey, sometimes (12) with...</t>
+          <t>...to roadside plantings. Cities also tend to use fewer pesticides than agricultural areas, (11) which can be harmful to bee populations. Urban bees have been found to produce high-quality honey, sometimes...</t>
         </is>
       </c>
       <c r="E45" s="3" t="inlineStr">
         <is>
-          <t>...(11) which can be harmful to bee populations. Urban bees have been found to produce high-quality honey, sometimes (12) with unique flavours reflecting the variety of flowers in their environment. Many cities now encourage urban...</t>
+          <t>...which can be harmful to bee populations. Urban bees have been found to produce high-quality honey, sometimes (12) with unique flavours reflecting the variety of flowers in their environment. Many cities now encourage urban...</t>
         </is>
       </c>
       <c r="F45" s="3" t="inlineStr">
@@ -6096,7 +6098,7 @@
         </is>
       </c>
     </row>
-    <row r="46" ht="60" customHeight="1">
+    <row r="46">
       <c r="A46" s="2" t="n">
         <v>45</v>
       </c>
@@ -6112,12 +6114,12 @@
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>...of debris larger than 10 centimetres currently orbiting Earth, along with millions of smaller fragments that are (11) too small to track but still dangerous. The main danger is (12) that space debris travels at incredibly high speeds –...</t>
+          <t>...of debris larger than 10 centimetres currently orbiting Earth, along with millions of smaller fragments that are (11) too small to track but still dangerous. The main danger is...</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>...along with millions of smaller fragments that are (11) too small to track but still dangerous. The main danger is (12) that space debris travels at incredibly high speeds – up to 28,000 kilometres per hour. At these velocities, even a...</t>
+          <t>...too small to track but still dangerous. The main danger is (12) that space debris travels at incredibly high speeds – up to 28,000 kilometres per hour. At these velocities, even a...</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
@@ -6221,18 +6223,18 @@
         </is>
       </c>
     </row>
-    <row r="47" ht="60" customHeight="1">
+    <row r="47">
       <c r="A47" s="3" t="n">
         <v>46</v>
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>...and emotional responses that music triggers. Studies have shown that listening to music activates multiple areas (9) of the brain simultaneously, including regions associated with emotion, memory, and movement. This may explain (10)...</t>
+          <t>...and emotional responses that music triggers. Studies have shown that listening to music activates multiple areas (9) of the brain simultaneously, including regions associated with emotion, memory, and movement. This may explain...</t>
         </is>
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>...(9) of the brain simultaneously, including regions associated with emotion, memory, and movement. This may explain (10) why certain songs can instantly transport us back to specific moments in our lives. The emotional power of music is...</t>
+          <t>...of the brain simultaneously, including regions associated with emotion, memory, and movement. This may explain (10) why certain songs can instantly transport us back to specific moments in our lives. The emotional power of music is...</t>
         </is>
       </c>
       <c r="D47" s="3" t="inlineStr">
@@ -6242,22 +6244,22 @@
       </c>
       <c r="E47" s="3" t="inlineStr">
         <is>
-          <t>...the span of a single composition. Music can also have practical benefits. Research indicates that students who study (12) while listening to baroque music perform better on tests, a phenomenon known as the 'Mozart effect', although (13) the...</t>
+          <t>...the span of a single composition. Music can also have practical benefits. Research indicates that students who study (12) while listening to baroque music perform better on tests, a phenomenon known as the 'Mozart effect', although...</t>
         </is>
       </c>
       <c r="F47" s="3" t="inlineStr">
         <is>
-          <t>...(12) while listening to baroque music perform better on tests, a phenomenon known as the 'Mozart effect', although (13) the extent of this effect remains debated. Hospitals use music therapy to help patients manage pain and anxiety....</t>
+          <t>...while listening to baroque music perform better on tests, a phenomenon known as the 'Mozart effect', although (13) the extent of this effect remains debated. Hospitals use music therapy to help patients manage pain and anxiety....</t>
         </is>
       </c>
       <c r="G47" s="3" t="inlineStr">
         <is>
-          <t>...effect remains debated. Hospitals use music therapy to help patients manage pain and anxiety. Athletes often listen (14) to energising music before competitions to boost motivation and performance. Scientists have (15) yet to fully explain...</t>
+          <t>...effect remains debated. Hospitals use music therapy to help patients manage pain and anxiety. Athletes often listen (14) to energising music before competitions to boost motivation and performance. Scientists have...</t>
         </is>
       </c>
       <c r="H47" s="3" t="inlineStr">
         <is>
-          <t>...often listen (14) to energising music before competitions to boost motivation and performance. Scientists have (15) yet to fully explain why humans respond so deeply to music. Some scientists believe musical ability evolved alongside...</t>
+          <t>...to energising music before competitions to boost motivation and performance. Scientists have (15) yet to fully explain why humans respond so deeply to music. Some scientists believe musical ability evolved alongside...</t>
         </is>
       </c>
       <c r="I47" s="3" t="inlineStr">
@@ -6346,7 +6348,7 @@
         </is>
       </c>
     </row>
-    <row r="48" ht="60" customHeight="1">
+    <row r="48">
       <c r="A48" s="2" t="n">
         <v>47</v>
       </c>
@@ -6471,7 +6473,7 @@
         </is>
       </c>
     </row>
-    <row r="49" ht="60" customHeight="1">
+    <row r="49">
       <c r="A49" s="3" t="n">
         <v>48</v>
       </c>
@@ -6596,7 +6598,7 @@
         </is>
       </c>
     </row>
-    <row r="50" ht="60" customHeight="1">
+    <row r="50">
       <c r="A50" s="2" t="n">
         <v>49</v>
       </c>
@@ -6622,22 +6624,22 @@
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>...importance of dark skies. Hotels and tour operators now offer specialised packages that include stargazing sessions (13) led by expert astronomers, telescope viewing, and photography workshops. The movement has also raised awareness (14)...</t>
+          <t>...importance of dark skies. Hotels and tour operators now offer specialised packages that include stargazing sessions (13) led by expert astronomers, telescope viewing, and photography workshops. The movement has also raised awareness...</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>...(13) led by expert astronomers, telescope viewing, and photography workshops. The movement has also raised awareness (14) about the environmental impacts of light pollution. Excessive artificial lighting affects wildlife, disrupts...</t>
+          <t>...led by expert astronomers, telescope viewing, and photography workshops. The movement has also raised awareness (14) about the environmental impacts of light pollution. Excessive artificial lighting affects wildlife, disrupts...</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr">
         <is>
-          <t>...energy. Many cities are now adopting better lighting practices, using shielded fixtures that direct light downward (15) rather than into the sky. International Dark Sky Association certifies locations based (16) on their sky quality and...</t>
+          <t>...energy. Many cities are now adopting better lighting practices, using shielded fixtures that direct light downward (15) rather than into the sky. International Dark Sky Association certifies locations based...</t>
         </is>
       </c>
       <c r="I50" s="2" t="inlineStr">
         <is>
-          <t>...that direct light downward (15) rather than into the sky. International Dark Sky Association certifies locations based (16) on their sky quality and commitment to reducing light pollution. As awareness grows, protecting dark skies is becoming...</t>
+          <t>...rather than into the sky. International Dark Sky Association certifies locations based (16) on their sky quality and commitment to reducing light pollution. As awareness grows, protecting dark skies is becoming...</t>
         </is>
       </c>
       <c r="J50" s="2" t="inlineStr">
@@ -6721,7 +6723,7 @@
         </is>
       </c>
     </row>
-    <row r="51" ht="60" customHeight="1">
+    <row r="51">
       <c r="A51" s="3" t="n">
         <v>50</v>
       </c>

</xml_diff>